<commit_message>
product image urls added
</commit_message>
<xml_diff>
--- a/yuva_store_data_updated.xlsx
+++ b/yuva_store_data_updated.xlsx
@@ -801,7 +801,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI3"/>
+  <dimension ref="A1:AJ4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -839,6 +839,7 @@
     <col width="16" customWidth="1" min="33" max="33"/>
     <col width="14" customWidth="1" min="34" max="34"/>
     <col width="50" customWidth="1" min="35" max="35"/>
+    <col width="50" customWidth="1" min="36" max="36"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1017,6 +1018,11 @@
           <t>Comma-separated usage tag slugs e.g. gaming,coding</t>
         </is>
       </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>Comma or newline separated image URLs (Drive links OK). First = primary</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1192,6 +1198,11 @@
       <c r="AI2" s="2" t="inlineStr">
         <is>
           <t>usage_tag_slugs</t>
+        </is>
+      </c>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>image_urls</t>
         </is>
       </c>
     </row>
@@ -1369,6 +1380,188 @@
       <c r="AI3" s="3" t="inlineStr">
         <is>
           <t>business,coding</t>
+        </is>
+      </c>
+      <c r="AJ3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>HP Pavilion 15</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>hp-pavilion-15</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>HP-PAV-15</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>laptops</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>27999.00</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>34000.00</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Intel Core i5 11th Gen</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>8GB DDR4</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>512GB NVMe SSD</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>15.6-inch Full HD</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>Intel Iris Xe</t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="inlineStr">
+        <is>
+          <t>Windows 11 Home</t>
+        </is>
+      </c>
+      <c r="P4" s="4" t="inlineStr">
+        <is>
+          <t>3-Cell 41Wh</t>
+        </is>
+      </c>
+      <c r="Q4" s="4" t="inlineStr">
+        <is>
+          <t>1.75 kg</t>
+        </is>
+      </c>
+      <c r="R4" s="4" t="inlineStr">
+        <is>
+          <t>USB-A x2, Type-C x1, HDMI x1</t>
+        </is>
+      </c>
+      <c r="S4" s="4" t="inlineStr">
+        <is>
+          <t>Wi-Fi 6</t>
+        </is>
+      </c>
+      <c r="T4" s="4" t="inlineStr">
+        <is>
+          <t>Bluetooth 5.1</t>
+        </is>
+      </c>
+      <c r="U4" s="4" t="inlineStr">
+        <is>
+          <t>Everyday performance laptop in great condition.</t>
+        </is>
+      </c>
+      <c r="V4" s="4" t="inlineStr">
+        <is>
+          <t>Intel i5 11th Gen
+8GB RAM &amp; 512GB SSD</t>
+        </is>
+      </c>
+      <c r="W4" s="4" t="inlineStr">
+        <is>
+          <t>40+ Quality Checks Passed</t>
+        </is>
+      </c>
+      <c r="X4" s="4" t="inlineStr">
+        <is>
+          <t>Display Checked
+Battery Health &gt; 90%
+Sound &amp; Mic Tested</t>
+        </is>
+      </c>
+      <c r="Y4" s="4" t="inlineStr">
+        <is>
+          <t>6 Months Warranty Included</t>
+        </is>
+      </c>
+      <c r="Z4" s="4" t="inlineStr">
+        <is>
+          <t>Covers internal components and adapter replacement.</t>
+        </is>
+      </c>
+      <c r="AA4" s="4" t="inlineStr">
+        <is>
+          <t>350+ Service Centers</t>
+        </is>
+      </c>
+      <c r="AB4" s="4" t="inlineStr">
+        <is>
+          <t>6 Months Warranty</t>
+        </is>
+      </c>
+      <c r="AC4" s="4" t="inlineStr">
+        <is>
+          <t>14 Days Return</t>
+        </is>
+      </c>
+      <c r="AD4" s="4" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AE4" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AF4" s="4" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AG4" s="4" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AH4" s="4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AI4" s="4" t="inlineStr">
+        <is>
+          <t>business,coding</t>
+        </is>
+      </c>
+      <c r="AJ4" s="4" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1W5xzHAfBIWVZRnPNepp7kpBLDJoCiMBe/view?usp=sharing, https://drive.google.com/file/d/1bgGAsruTtcGVU5VTJ-FqHOCaCgZSOhaQ/view?usp=sharing</t>
         </is>
       </c>
     </row>

</xml_diff>